<commit_message>
Formandos: colar a coluna NOME tal como vem das listas do IEFP
As listas do IEFP trazem o nome completo numa so coluna e em
maiusculas. Em vez de partir nomes a mao, o Repo faz isso ao carregar:
com o Apelido em branco, o primeiro nome vai para o Nome e o resto para
o Apelido; um nome todo em maiusculas (ou todo em minusculas) passa a
"Ana Margarida dos Santos Mendes". Um nome ja escrito com maiusculas e
minusculas fica como esta. O modelo diz isto na nota do Nome e num
passo novo das instrucoes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/repo/modelo-formandos.xlsx
+++ b/repo/modelo-formandos.xlsx
@@ -31,7 +31,7 @@
             <sz val="9"/>
             <rFont val="Arial"/>
           </rPr>
-          <t>Obrigatório. Só o primeiro nome, ou os nomes próprios.</t>
+          <t>Obrigatório. Podes colar aqui o nome completo, mesmo em maiúsculas, e deixar o Apelido em branco: o Repo parte-o e acerta-o ao carregar.</t>
         </r>
       </text>
     </comment>
@@ -117,7 +117,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="31">
   <si>
     <t>Nome</t>
   </si>
@@ -182,10 +182,13 @@
     <t>4. Para várias pessoas do mesmo curso, preenche o Curso, a Entidade e as datas na primeira linha e arrasta para baixo.</t>
   </si>
   <si>
-    <t>5. Pode ser uma formação por ficheiro ou todas no mesmo. Os dois funcionam.</t>
+    <t>5. Se a lista tem o nome completo numa só coluna (como as do IEFP), cola-o todo no Nome e deixa o Apelido em branco. Maiúsculas não fazem mal: o Repo parte o nome e acerta-o ao carregar.</t>
   </si>
   <si>
-    <t>6. Grava como .xlsx e carrega no Repo, em Formandos.</t>
+    <t>6. Pode ser uma formação por ficheiro ou todas no mesmo. Os dois funcionam.</t>
+  </si>
+  <si>
+    <t>7. Grava como .xlsx e carrega no Repo, em Formandos.</t>
   </si>
   <si>
     <t>Obrigatórios: Nome, Email, Curso, Entidade. O resto ajuda, mas pode ficar em branco.</t>
@@ -14777,7 +14780,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I17"/>
+  <dimension ref="B2:I18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -14873,96 +14876,108 @@
       <c r="H9" s="9"/>
       <c r="I9" s="9"/>
     </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B11" s="5" t="s">
+    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B10" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
-    </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B13" s="5" t="s">
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+      <c r="H10" s="9"/>
+      <c r="I10" s="9"/>
+    </row>
+    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B12" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="5"/>
+      <c r="I12" s="5"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
+      <c r="I14" s="5"/>
+    </row>
+    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B15" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="C15" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="D15" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="E14" s="10" t="s">
+      <c r="E15" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="F14" s="10" t="s">
+      <c r="F15" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="G14" s="10" t="s">
+      <c r="G15" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="H14" s="10" t="s">
+      <c r="H15" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="I14" s="10" t="s">
+      <c r="I15" s="10" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B15" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="C15" s="11" t="s">
+    <row r="16" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B16" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="11" t="s">
+      <c r="C16" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="E15" s="11" t="s">
+      <c r="D16" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="E16" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="F15" s="11" t="s">
+      <c r="F16" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="G15" s="12">
+      <c r="G16" s="12">
         <v>46279</v>
       </c>
-      <c r="H15" s="12">
+      <c r="H16" s="12">
         <v>46325</v>
       </c>
-      <c r="I15" s="11" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B17" s="7" t="s">
+      <c r="I16" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
-      <c r="G17" s="7"/>
-      <c r="H17" s="7"/>
-      <c r="I17" s="7"/>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B18" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="7"/>
+      <c r="H18" s="7"/>
+      <c r="I18" s="7"/>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="B2:I2"/>
     <mergeCell ref="B4:I4"/>
     <mergeCell ref="B5:I5"/>
@@ -14970,9 +14985,10 @@
     <mergeCell ref="B7:I7"/>
     <mergeCell ref="B8:I8"/>
     <mergeCell ref="B9:I9"/>
-    <mergeCell ref="B11:I11"/>
-    <mergeCell ref="B13:I13"/>
-    <mergeCell ref="B17:I17"/>
+    <mergeCell ref="B10:I10"/>
+    <mergeCell ref="B12:I12"/>
+    <mergeCell ref="B14:I14"/>
+    <mergeCell ref="B18:I18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Formandos: as turmas gerem-se pelo mes
O curso tem sempre o mesmo nome; o que distingue uma turma de outra e o
mes ("Turma Janeiro 2026"). O Repo passa a guardar o primeiro dia do
mes, seja qual for o dia escrito - "12/01/2026" num ficheiro e "01/2026"
noutro sao a mesma turma - e a mostrar "janeiro 2026" ou "setembro a
outubro 2026" em vez de datas ao dia.

Aceita uma data do Excel, dd/mm/aaaa, mm/aaaa, aaaa-mm, "janeiro 2026"
e "jan/2026". As colunas Inicio e Fim do modelo mostram o mes e a nota
diz que basta o mes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/repo/modelo-formandos.xlsx
+++ b/repo/modelo-formandos.xlsx
@@ -86,7 +86,7 @@
             <sz val="9"/>
             <rFont val="Arial"/>
           </rPr>
-          <t>Data de início da formação, dd/mm/aaaa.</t>
+          <t>O mês da turma. Basta o mês: escreve 01/2026 ou janeiro 2026.</t>
         </r>
       </text>
     </comment>
@@ -97,7 +97,7 @@
             <sz val="9"/>
             <rFont val="Arial"/>
           </rPr>
-          <t>Data de fim. Opcional.</t>
+          <t>Opcional. O mês em que acabou, se não for o mesmo do início.</t>
         </r>
       </text>
     </comment>
@@ -217,7 +217,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="164" formatCode="mmmm yyyy"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -670,7 +670,7 @@
     <col min="3" max="3" width="32" customWidth="1"/>
     <col min="4" max="4" width="30" customWidth="1"/>
     <col min="5" max="5" width="22" customWidth="1"/>
-    <col min="6" max="7" width="12" customWidth="1"/>
+    <col min="6" max="7" width="16" customWidth="1"/>
     <col min="8" max="8" width="36" customWidth="1"/>
   </cols>
   <sheetData>
@@ -14788,7 +14788,7 @@
     <col min="4" max="4" width="28" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
     <col min="6" max="6" width="20" customWidth="1"/>
-    <col min="7" max="8" width="12" customWidth="1"/>
+    <col min="7" max="8" width="16" customWidth="1"/>
     <col min="9" max="9" width="22" customWidth="1"/>
   </cols>
   <sheetData>
@@ -14955,10 +14955,10 @@
         <v>11</v>
       </c>
       <c r="G16" s="12">
-        <v>46279</v>
+        <v>46266</v>
       </c>
       <c r="H16" s="12">
-        <v>46325</v>
+        <v>46296</v>
       </c>
       <c r="I16" s="11" t="s">
         <v>29</v>

</xml_diff>